<commit_message>
/HARDWARE: corrected schematics naming
</commit_message>
<xml_diff>
--- a/Hardware/production/positions.xlsx
+++ b/Hardware/production/positions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saleh\Desktop\Saleh Uni\sem 7\senior year project\Flight Controller\Hardware\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA6B7F8-C0D4-4308-8802-3505BC4F6993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E695700F-6AD7-4D21-9AF3-ABCA8536A634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="720" windowWidth="19200" windowHeight="11170" xr2:uid="{6F0F2AF3-BE7C-4435-8EF3-B97DB954307E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{EF06F55D-5B1F-40CB-A247-AAC625F064EC}"/>
   </bookViews>
   <sheets>
     <sheet name="positions" sheetId="1" r:id="rId1"/>
@@ -1392,11 +1392,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AF5571C-5D62-44DB-9E1C-A3DF3CCED614}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA64EEC3-A27F-418C-B928-4338AB0E5B9E}">
   <dimension ref="A1:E165"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -1472,7 +1473,7 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>144.7525</v>
+        <v>144.5575</v>
       </c>
       <c r="C5">
         <v>-91.537499999999994</v>
@@ -1489,7 +1490,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>144.7525</v>
+        <v>144.5575</v>
       </c>
       <c r="C6">
         <v>-92.837500000000006</v>
@@ -1883,7 +1884,7 @@
         <v>122.15</v>
       </c>
       <c r="C29">
-        <v>-110.39</v>
+        <v>-110.14</v>
       </c>
       <c r="D29">
         <v>270</v>
@@ -2036,7 +2037,7 @@
         <v>132.34</v>
       </c>
       <c r="C38">
-        <v>-85.23</v>
+        <v>-85.46</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -2053,7 +2054,7 @@
         <v>132.38</v>
       </c>
       <c r="C39">
-        <v>-86.74</v>
+        <v>-86.98</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -2104,7 +2105,7 @@
         <v>131.41999999999999</v>
       </c>
       <c r="C42">
-        <v>-88.41</v>
+        <v>-89.17</v>
       </c>
       <c r="D42">
         <v>90</v>
@@ -2121,7 +2122,7 @@
         <v>132.84</v>
       </c>
       <c r="C43">
-        <v>-87.95</v>
+        <v>-88.24</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -2696,7 +2697,7 @@
         <v>82</v>
       </c>
       <c r="B77">
-        <v>144.56</v>
+        <v>144.46714600000001</v>
       </c>
       <c r="C77">
         <v>-96.18</v>
@@ -2886,7 +2887,7 @@
         <v>124.14</v>
       </c>
       <c r="C88">
-        <v>-99.65</v>
+        <v>-99.22</v>
       </c>
       <c r="D88">
         <v>0</v>
@@ -2903,7 +2904,7 @@
         <v>124.02</v>
       </c>
       <c r="C89">
-        <v>-109.96</v>
+        <v>-109.66</v>
       </c>
       <c r="D89">
         <v>180</v>
@@ -2920,7 +2921,7 @@
         <v>122.17</v>
       </c>
       <c r="C90">
-        <v>-99.24</v>
+        <v>-98.81</v>
       </c>
       <c r="D90">
         <v>90</v>
@@ -2971,7 +2972,7 @@
         <v>130.41999999999999</v>
       </c>
       <c r="C93">
-        <v>-88.39</v>
+        <v>-89.15</v>
       </c>
       <c r="D93">
         <v>270</v>
@@ -4161,7 +4162,7 @@
         <v>124.07</v>
       </c>
       <c r="C163">
-        <v>-104.88500000000001</v>
+        <v>-104.47499999999999</v>
       </c>
       <c r="D163">
         <v>270</v>

</xml_diff>